<commit_message>
Updated product strings for LST geo data
</commit_message>
<xml_diff>
--- a/data/cci/cci-product.xlsx
+++ b/data/cci/cci-product.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stfc365-my.sharepoint.com/personal/alison_waterfall_stfc_ac_uk/Documents/Documents/GitHub/cci-vocabularies/data/cci/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="13_ncr:1_{8698D110-CEA0-44F5-A4A0-4B424D64BB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84D3283B-EF48-4A58-82A1-9A3249C51EF6}"/>
+  <xr:revisionPtr revIDLastSave="142" documentId="13_ncr:1_{8698D110-CEA0-44F5-A4A0-4B424D64BB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8AE1811C-B940-4021-823D-619C586D6182}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{04DF87AA-227F-E848-BF0E-6E7C9BB1D368}"/>
+    <workbookView xWindow="38280" yWindow="-60" windowWidth="38640" windowHeight="21120" xr2:uid="{04DF87AA-227F-E848-BF0E-6E7C9BB1D368}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="590">
   <si>
     <t>URI</t>
   </si>
@@ -1733,6 +1733,63 @@
   </si>
   <si>
     <t>prod_s1bIw</t>
+  </si>
+  <si>
+    <t>prod_goes1213Mon</t>
+  </si>
+  <si>
+    <t>GOES12_13-0.05deg_1MONTHLY</t>
+  </si>
+  <si>
+    <t>prod_goes1213</t>
+  </si>
+  <si>
+    <t>GOES12_13-0.05deg</t>
+  </si>
+  <si>
+    <t>prod_goes16</t>
+  </si>
+  <si>
+    <t>GOES16-0.05deg</t>
+  </si>
+  <si>
+    <t>prod_goes16Mon</t>
+  </si>
+  <si>
+    <t>GOES16-0.05deg_1MONTHLY</t>
+  </si>
+  <si>
+    <t>prod_mtsatMon</t>
+  </si>
+  <si>
+    <t>MTSAT1_2-0.05deg_1MONTHLY</t>
+  </si>
+  <si>
+    <t>prod_mtsat</t>
+  </si>
+  <si>
+    <t>MTSAT1_2-0.05deg</t>
+  </si>
+  <si>
+    <t>prod_hmwr8Mon</t>
+  </si>
+  <si>
+    <t>HMWR8-0.05deg_1MONTHLY</t>
+  </si>
+  <si>
+    <t>prod_hmwr8</t>
+  </si>
+  <si>
+    <t>HMWR8-0.05deg</t>
+  </si>
+  <si>
+    <t>prod_hmwr9Mon</t>
+  </si>
+  <si>
+    <t>HMWR9-0.05deg_1MONTHLY</t>
+  </si>
+  <si>
+    <t>HMWR9-0.05deg</t>
   </si>
 </sst>
 </file>
@@ -2021,10 +2078,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2360,19 +2413,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A059DA7-785A-874C-8D00-32DC40CC12B7}">
-  <dimension ref="A1:AMC242"/>
-  <sheetFormatPr defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AMC252"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.26953125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="23.453125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="50.453125" style="2" customWidth="1"/>
-    <col min="5" max="1016" width="10.7265625" style="2" customWidth="1"/>
-    <col min="1017" max="1017" width="13.26953125" style="2" customWidth="1"/>
-    <col min="1018" max="1018" width="10.7265625" customWidth="1"/>
+    <col min="1" max="1" width="36.28515625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="50.42578125" style="2" customWidth="1"/>
+    <col min="5" max="1016" width="10.7109375" style="2" customWidth="1"/>
+    <col min="1017" max="1017" width="13.28515625" style="2" customWidth="1"/>
+    <col min="1018" max="1018" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2389,7 +2442,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -2400,7 +2453,7 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
@@ -2413,7 +2466,7 @@
       </c>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
@@ -2424,7 +2477,7 @@
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
@@ -2435,7 +2488,7 @@
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -2446,7 +2499,7 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
@@ -2457,7 +2510,7 @@
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -2468,7 +2521,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -2479,7 +2532,7 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2490,7 +2543,7 @@
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>24</v>
       </c>
@@ -2501,7 +2554,7 @@
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>26</v>
       </c>
@@ -2512,7 +2565,7 @@
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>28</v>
       </c>
@@ -2523,7 +2576,7 @@
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>30</v>
       </c>
@@ -2534,7 +2587,7 @@
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>32</v>
       </c>
@@ -2545,7 +2598,7 @@
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>34</v>
       </c>
@@ -2556,7 +2609,7 @@
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
     </row>
-    <row r="17" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>36</v>
       </c>
@@ -2569,7 +2622,7 @@
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>39</v>
       </c>
@@ -2580,7 +2633,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>41</v>
       </c>
@@ -2591,7 +2644,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>43</v>
       </c>
@@ -2602,7 +2655,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
     </row>
-    <row r="21" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>45</v>
       </c>
@@ -2613,7 +2666,7 @@
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
     </row>
-    <row r="22" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>47</v>
       </c>
@@ -2624,7 +2677,7 @@
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
     </row>
-    <row r="23" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>49</v>
       </c>
@@ -2635,7 +2688,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
     </row>
-    <row r="24" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>51</v>
       </c>
@@ -2648,7 +2701,7 @@
       </c>
       <c r="E24" s="3"/>
     </row>
-    <row r="25" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>54</v>
       </c>
@@ -2659,7 +2712,7 @@
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
     </row>
-    <row r="26" spans="1:64" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:64" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>56</v>
       </c>
@@ -2729,7 +2782,7 @@
       <c r="BK26" s="2"/>
       <c r="BL26" s="2"/>
     </row>
-    <row r="27" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>58</v>
       </c>
@@ -2740,7 +2793,7 @@
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>60</v>
       </c>
@@ -2751,7 +2804,7 @@
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
     </row>
-    <row r="29" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>62</v>
       </c>
@@ -2762,7 +2815,7 @@
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>64</v>
       </c>
@@ -2773,7 +2826,7 @@
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
     </row>
-    <row r="31" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>66</v>
       </c>
@@ -2784,7 +2837,7 @@
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
     </row>
-    <row r="32" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>68</v>
       </c>
@@ -2795,7 +2848,7 @@
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
     </row>
-    <row r="33" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>70</v>
       </c>
@@ -2806,7 +2859,7 @@
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
     </row>
-    <row r="34" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>72</v>
       </c>
@@ -2817,7 +2870,7 @@
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
     </row>
-    <row r="35" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>74</v>
       </c>
@@ -3781,7 +3834,7 @@
       <c r="AMB35"/>
       <c r="AMC35"/>
     </row>
-    <row r="36" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>76</v>
       </c>
@@ -4745,7 +4798,7 @@
       <c r="AMB36"/>
       <c r="AMC36"/>
     </row>
-    <row r="37" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>78</v>
       </c>
@@ -5709,7 +5762,7 @@
       <c r="AMB37"/>
       <c r="AMC37"/>
     </row>
-    <row r="38" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>80</v>
       </c>
@@ -6673,7 +6726,7 @@
       <c r="AMB38"/>
       <c r="AMC38"/>
     </row>
-    <row r="39" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>82</v>
       </c>
@@ -6684,7 +6737,7 @@
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
     </row>
-    <row r="40" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>84</v>
       </c>
@@ -6697,7 +6750,7 @@
       </c>
       <c r="E40" s="3"/>
     </row>
-    <row r="41" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>87</v>
       </c>
@@ -6708,7 +6761,7 @@
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
     </row>
-    <row r="42" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>89</v>
       </c>
@@ -6719,7 +6772,7 @@
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
     </row>
-    <row r="43" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>91</v>
       </c>
@@ -6732,7 +6785,7 @@
       </c>
       <c r="E43" s="3"/>
     </row>
-    <row r="44" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>94</v>
       </c>
@@ -6743,7 +6796,7 @@
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
     </row>
-    <row r="45" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>96</v>
       </c>
@@ -6756,7 +6809,7 @@
       </c>
       <c r="E45"/>
     </row>
-    <row r="46" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>99</v>
       </c>
@@ -6767,7 +6820,7 @@
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
     </row>
-    <row r="47" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>101</v>
       </c>
@@ -6778,7 +6831,7 @@
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
     </row>
-    <row r="48" spans="1:1017" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:1017" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>103</v>
       </c>
@@ -6791,7 +6844,7 @@
       </c>
       <c r="E48" s="3"/>
     </row>
-    <row r="49" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>106</v>
       </c>
@@ -6802,7 +6855,7 @@
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
     </row>
-    <row r="50" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>108</v>
       </c>
@@ -6813,7 +6866,7 @@
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
     </row>
-    <row r="51" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>110</v>
       </c>
@@ -6824,7 +6877,7 @@
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
     </row>
-    <row r="52" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>112</v>
       </c>
@@ -6835,7 +6888,7 @@
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
     </row>
-    <row r="53" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>114</v>
       </c>
@@ -6846,7 +6899,7 @@
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
     </row>
-    <row r="54" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:64" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>116</v>
       </c>
@@ -6859,7 +6912,7 @@
       </c>
       <c r="E54" s="3"/>
     </row>
-    <row r="55" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>119</v>
       </c>
@@ -6872,7 +6925,7 @@
       </c>
       <c r="E55" s="3"/>
     </row>
-    <row r="56" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>122</v>
       </c>
@@ -6885,7 +6938,7 @@
       </c>
       <c r="E56" s="3"/>
     </row>
-    <row r="57" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>125</v>
       </c>
@@ -6898,7 +6951,7 @@
       </c>
       <c r="E57" s="3"/>
     </row>
-    <row r="58" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>128</v>
       </c>
@@ -6911,7 +6964,7 @@
       </c>
       <c r="E58" s="3"/>
     </row>
-    <row r="59" spans="1:64" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:64" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>131</v>
       </c>
@@ -6981,7 +7034,7 @@
       <c r="BK59" s="2"/>
       <c r="BL59" s="2"/>
     </row>
-    <row r="60" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>133</v>
       </c>
@@ -6992,7 +7045,7 @@
       <c r="D60" s="3"/>
       <c r="E60" s="3"/>
     </row>
-    <row r="61" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>135</v>
       </c>
@@ -7003,7 +7056,7 @@
       <c r="D61" s="3"/>
       <c r="E61" s="3"/>
     </row>
-    <row r="62" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>137</v>
       </c>
@@ -7014,7 +7067,7 @@
       <c r="D62" s="3"/>
       <c r="E62" s="3"/>
     </row>
-    <row r="63" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>139</v>
       </c>
@@ -7027,7 +7080,7 @@
       </c>
       <c r="E63" s="3"/>
     </row>
-    <row r="64" spans="1:64" ht="29" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:64" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>142</v>
       </c>
@@ -7040,7 +7093,7 @@
       </c>
       <c r="E64" s="3"/>
     </row>
-    <row r="65" spans="1:64" ht="29" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:64" ht="30" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
         <v>145</v>
       </c>
@@ -7053,7 +7106,7 @@
       </c>
       <c r="E65" s="3"/>
     </row>
-    <row r="66" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>148</v>
       </c>
@@ -7066,7 +7119,7 @@
       </c>
       <c r="E66" s="3"/>
     </row>
-    <row r="67" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>151</v>
       </c>
@@ -7077,7 +7130,7 @@
       <c r="D67" s="3"/>
       <c r="E67" s="3"/>
     </row>
-    <row r="68" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>153</v>
       </c>
@@ -7088,7 +7141,7 @@
       <c r="D68" s="3"/>
       <c r="E68" s="3"/>
     </row>
-    <row r="69" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>155</v>
       </c>
@@ -7099,7 +7152,7 @@
       <c r="D69" s="3"/>
       <c r="E69" s="3"/>
     </row>
-    <row r="70" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>157</v>
       </c>
@@ -7110,7 +7163,7 @@
       <c r="D70" s="3"/>
       <c r="E70" s="3"/>
     </row>
-    <row r="71" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>159</v>
       </c>
@@ -7121,7 +7174,7 @@
       <c r="D71" s="3"/>
       <c r="E71" s="3"/>
     </row>
-    <row r="72" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>161</v>
       </c>
@@ -7132,7 +7185,7 @@
       <c r="D72" s="3"/>
       <c r="E72" s="3"/>
     </row>
-    <row r="73" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>163</v>
       </c>
@@ -7143,7 +7196,7 @@
       <c r="D73" s="3"/>
       <c r="E73" s="3"/>
     </row>
-    <row r="74" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>165</v>
       </c>
@@ -7154,7 +7207,7 @@
       <c r="D74" s="3"/>
       <c r="E74" s="3"/>
     </row>
-    <row r="75" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>167</v>
       </c>
@@ -7167,7 +7220,7 @@
       </c>
       <c r="E75" s="3"/>
     </row>
-    <row r="76" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>169</v>
       </c>
@@ -7178,7 +7231,7 @@
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
     </row>
-    <row r="77" spans="1:64" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:64" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>171</v>
       </c>
@@ -7248,7 +7301,7 @@
       <c r="BK77" s="2"/>
       <c r="BL77" s="2"/>
     </row>
-    <row r="78" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
         <v>173</v>
       </c>
@@ -7259,7 +7312,7 @@
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
     </row>
-    <row r="79" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>175</v>
       </c>
@@ -7270,7 +7323,7 @@
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
     </row>
-    <row r="80" spans="1:64" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
         <v>177</v>
       </c>
@@ -7281,7 +7334,7 @@
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>179</v>
       </c>
@@ -7292,7 +7345,7 @@
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>181</v>
       </c>
@@ -7305,7 +7358,7 @@
       </c>
       <c r="E82" s="3"/>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>184</v>
       </c>
@@ -7318,7 +7371,7 @@
       </c>
       <c r="E83" s="3"/>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>187</v>
       </c>
@@ -7329,7 +7382,7 @@
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>189</v>
       </c>
@@ -7340,7 +7393,7 @@
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>191</v>
       </c>
@@ -7353,7 +7406,7 @@
       </c>
       <c r="E86" s="3"/>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>194</v>
       </c>
@@ -7366,7 +7419,7 @@
       </c>
       <c r="E87" s="3"/>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>197</v>
       </c>
@@ -7379,7 +7432,7 @@
       </c>
       <c r="E88" s="3"/>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>200</v>
       </c>
@@ -7392,7 +7445,7 @@
       </c>
       <c r="E89" s="3"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>203</v>
       </c>
@@ -7403,7 +7456,7 @@
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
         <v>205</v>
       </c>
@@ -7414,7 +7467,7 @@
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
         <v>207</v>
       </c>
@@ -7425,7 +7478,7 @@
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
         <v>209</v>
       </c>
@@ -7436,7 +7489,7 @@
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>211</v>
       </c>
@@ -7449,7 +7502,7 @@
       </c>
       <c r="E94" s="3"/>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
         <v>214</v>
       </c>
@@ -7460,7 +7513,7 @@
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
         <v>216</v>
       </c>
@@ -7471,7 +7524,7 @@
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
         <v>218</v>
       </c>
@@ -7482,7 +7535,7 @@
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>220</v>
       </c>
@@ -7495,7 +7548,7 @@
       </c>
       <c r="E98" s="3"/>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
         <v>223</v>
       </c>
@@ -7506,7 +7559,7 @@
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
         <v>225</v>
       </c>
@@ -7517,7 +7570,7 @@
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
         <v>227</v>
       </c>
@@ -7528,7 +7581,7 @@
       <c r="D101" s="3"/>
       <c r="E101" s="3"/>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
         <v>229</v>
       </c>
@@ -7539,7 +7592,7 @@
       <c r="D102" s="3"/>
       <c r="E102" s="3"/>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
         <v>231</v>
       </c>
@@ -7552,7 +7605,7 @@
       </c>
       <c r="E103" s="3"/>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
         <v>234</v>
       </c>
@@ -7565,7 +7618,7 @@
       </c>
       <c r="E104" s="3"/>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
         <v>237</v>
       </c>
@@ -7576,7 +7629,7 @@
       <c r="D105" s="3"/>
       <c r="E105" s="3"/>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
         <v>239</v>
       </c>
@@ -7587,7 +7640,7 @@
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
         <v>241</v>
       </c>
@@ -7598,7 +7651,7 @@
       <c r="D107" s="3"/>
       <c r="E107" s="3"/>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
         <v>243</v>
       </c>
@@ -7609,7 +7662,7 @@
       <c r="D108" s="3"/>
       <c r="E108" s="3"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>245</v>
       </c>
@@ -7622,7 +7675,7 @@
       </c>
       <c r="E109" s="3"/>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>248</v>
       </c>
@@ -7633,7 +7686,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>251</v>
       </c>
@@ -7641,7 +7694,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>253</v>
       </c>
@@ -7652,7 +7705,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>256</v>
       </c>
@@ -7663,7 +7716,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>259</v>
       </c>
@@ -7674,7 +7727,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>262</v>
       </c>
@@ -7685,7 +7738,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>265</v>
       </c>
@@ -7696,7 +7749,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>268</v>
       </c>
@@ -7707,7 +7760,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>271</v>
       </c>
@@ -7718,7 +7771,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>274</v>
       </c>
@@ -7729,7 +7782,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>277</v>
       </c>
@@ -7740,7 +7793,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>280</v>
       </c>
@@ -7748,7 +7801,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>282</v>
       </c>
@@ -7756,7 +7809,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>284</v>
       </c>
@@ -7764,7 +7817,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>286</v>
       </c>
@@ -7772,7 +7825,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>288</v>
       </c>
@@ -7780,7 +7833,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>290</v>
       </c>
@@ -7791,7 +7844,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>293</v>
       </c>
@@ -7799,7 +7852,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>295</v>
       </c>
@@ -7807,7 +7860,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>297</v>
       </c>
@@ -7815,7 +7868,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>299</v>
       </c>
@@ -7823,7 +7876,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>301</v>
       </c>
@@ -7834,7 +7887,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>304</v>
       </c>
@@ -7845,7 +7898,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>307</v>
       </c>
@@ -7856,7 +7909,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>310</v>
       </c>
@@ -7867,7 +7920,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>313</v>
       </c>
@@ -7878,7 +7931,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>316</v>
       </c>
@@ -7889,7 +7942,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
         <v>319</v>
       </c>
@@ -7900,7 +7953,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>322</v>
       </c>
@@ -7911,7 +7964,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>325</v>
       </c>
@@ -7922,7 +7975,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>328</v>
       </c>
@@ -7933,7 +7986,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>331</v>
       </c>
@@ -7944,7 +7997,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>334</v>
       </c>
@@ -7955,7 +8008,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>337</v>
       </c>
@@ -7966,7 +8019,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>340</v>
       </c>
@@ -7977,7 +8030,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>343</v>
       </c>
@@ -7988,7 +8041,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>346</v>
       </c>
@@ -7999,7 +8052,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>349</v>
       </c>
@@ -8010,7 +8063,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>352</v>
       </c>
@@ -8021,7 +8074,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>355</v>
       </c>
@@ -8032,7 +8085,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>358</v>
       </c>
@@ -8043,7 +8096,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>361</v>
       </c>
@@ -8054,7 +8107,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>364</v>
       </c>
@@ -8065,7 +8118,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>367</v>
       </c>
@@ -8076,7 +8129,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>370</v>
       </c>
@@ -8087,7 +8140,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
         <v>373</v>
       </c>
@@ -8098,7 +8151,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>376</v>
       </c>
@@ -8109,7 +8162,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
         <v>379</v>
       </c>
@@ -8120,7 +8173,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>382</v>
       </c>
@@ -8131,7 +8184,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>385</v>
       </c>
@@ -8142,7 +8195,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
         <v>388</v>
       </c>
@@ -8153,7 +8206,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="161" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>391</v>
       </c>
@@ -8164,7 +8217,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="162" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>394</v>
       </c>
@@ -8175,7 +8228,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="163" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
         <v>397</v>
       </c>
@@ -8186,7 +8239,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>400</v>
       </c>
@@ -8197,7 +8250,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
         <v>403</v>
       </c>
@@ -8208,7 +8261,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
         <v>405</v>
       </c>
@@ -8219,7 +8272,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
         <v>407</v>
       </c>
@@ -8227,7 +8280,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>409</v>
       </c>
@@ -8235,7 +8288,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
         <v>411</v>
       </c>
@@ -8246,7 +8299,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
         <v>414</v>
       </c>
@@ -8257,7 +8310,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>417</v>
       </c>
@@ -8268,7 +8321,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
         <v>420</v>
       </c>
@@ -8279,7 +8332,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
         <v>423</v>
       </c>
@@ -8290,7 +8343,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
         <v>426</v>
       </c>
@@ -8301,7 +8354,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
         <v>429</v>
       </c>
@@ -8312,7 +8365,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
         <v>432</v>
       </c>
@@ -8323,7 +8376,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
         <v>435</v>
       </c>
@@ -8334,7 +8387,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
         <v>438</v>
       </c>
@@ -8342,7 +8395,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
         <v>440</v>
       </c>
@@ -8350,7 +8403,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
         <v>442</v>
       </c>
@@ -8358,7 +8411,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
         <v>444</v>
       </c>
@@ -8366,7 +8419,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
         <v>446</v>
       </c>
@@ -8374,7 +8427,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
         <v>448</v>
       </c>
@@ -8382,7 +8435,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
         <v>450</v>
       </c>
@@ -8390,7 +8443,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
         <v>452</v>
       </c>
@@ -8398,7 +8451,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
         <v>454</v>
       </c>
@@ -8406,7 +8459,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
         <v>456</v>
       </c>
@@ -8414,7 +8467,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
         <v>458</v>
       </c>
@@ -8422,7 +8475,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
         <v>460</v>
       </c>
@@ -8430,7 +8483,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
         <v>462</v>
       </c>
@@ -8438,7 +8491,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
         <v>464</v>
       </c>
@@ -8446,7 +8499,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
         <v>466</v>
       </c>
@@ -8454,7 +8507,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
         <v>468</v>
       </c>
@@ -8462,7 +8515,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
         <v>472</v>
       </c>
@@ -8470,7 +8523,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
         <v>473</v>
       </c>
@@ -8478,7 +8531,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
         <v>474</v>
       </c>
@@ -8489,7 +8542,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
         <v>475</v>
       </c>
@@ -8500,7 +8553,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
         <v>481</v>
       </c>
@@ -8508,7 +8561,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
         <v>482</v>
       </c>
@@ -8516,7 +8569,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
         <v>485</v>
       </c>
@@ -8524,7 +8577,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
         <v>486</v>
       </c>
@@ -8532,7 +8585,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
         <v>487</v>
       </c>
@@ -8540,7 +8593,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
         <v>488</v>
       </c>
@@ -8548,7 +8601,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
         <v>489</v>
       </c>
@@ -8556,7 +8609,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
         <v>496</v>
       </c>
@@ -8564,7 +8617,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
         <v>495</v>
       </c>
@@ -8572,7 +8625,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
         <v>499</v>
       </c>
@@ -8580,7 +8633,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>498</v>
       </c>
@@ -8588,7 +8641,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
         <v>502</v>
       </c>
@@ -8596,7 +8649,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>507</v>
       </c>
@@ -8604,7 +8657,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>508</v>
       </c>
@@ -8612,7 +8665,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
         <v>509</v>
       </c>
@@ -8620,7 +8673,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
         <v>510</v>
       </c>
@@ -8628,7 +8681,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
         <v>512</v>
       </c>
@@ -8636,7 +8689,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
         <v>514</v>
       </c>
@@ -8647,7 +8700,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
         <v>517</v>
       </c>
@@ -8655,7 +8708,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
         <v>519</v>
       </c>
@@ -8663,7 +8716,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
         <v>521</v>
       </c>
@@ -8671,7 +8724,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
         <v>523</v>
       </c>
@@ -8679,7 +8732,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
         <v>525</v>
       </c>
@@ -8687,7 +8740,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
         <v>526</v>
       </c>
@@ -8695,7 +8748,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
         <v>569</v>
       </c>
@@ -8703,7 +8756,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
         <v>570</v>
       </c>
@@ -8711,7 +8764,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
         <v>529</v>
       </c>
@@ -8719,7 +8772,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="225" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
         <v>530</v>
       </c>
@@ -8727,7 +8780,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="226" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
         <v>531</v>
       </c>
@@ -8735,7 +8788,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="227" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
         <v>535</v>
       </c>
@@ -8743,7 +8796,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="228" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A228" s="2" t="s">
         <v>538</v>
       </c>
@@ -8751,7 +8804,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="229" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A229" s="2" t="s">
         <v>540</v>
       </c>
@@ -8759,7 +8812,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="230" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A230" s="2" t="s">
         <v>542</v>
       </c>
@@ -8767,7 +8820,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="231" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
         <v>544</v>
       </c>
@@ -8775,7 +8828,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="232" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A232" s="2" t="s">
         <v>545</v>
       </c>
@@ -8783,7 +8836,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="233" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A233" s="2" t="s">
         <v>548</v>
       </c>
@@ -8791,7 +8844,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="234" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A234" s="2" t="s">
         <v>549</v>
       </c>
@@ -8799,7 +8852,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="235" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
         <v>559</v>
       </c>
@@ -8807,7 +8860,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="236" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A236" s="2" t="s">
         <v>560</v>
       </c>
@@ -8815,7 +8868,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="237" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A237" s="2" t="s">
         <v>561</v>
       </c>
@@ -8823,7 +8876,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="238" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A238" s="2" t="s">
         <v>562</v>
       </c>
@@ -8831,7 +8884,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="239" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A239" s="2" t="s">
         <v>563</v>
       </c>
@@ -8839,7 +8892,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="240" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A240" s="2" t="s">
         <v>564</v>
       </c>
@@ -8847,7 +8900,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="241" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A241" s="2" t="s">
         <v>565</v>
       </c>
@@ -8855,21 +8908,101 @@
         <v>557</v>
       </c>
     </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A242" s="2" t="s">
         <v>566</v>
       </c>
       <c r="B242" s="2" t="s">
         <v>558</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A243" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="B243" s="2" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A244" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="B244" s="2" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A245" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="B245" s="2" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A246" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="B246" s="2" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A247" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="B247" s="2" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A248" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="B248" s="2" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A249" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="B249" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A250" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="B250" s="2" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A251" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="B251" s="2" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A252" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="B252" s="2" t="s">
+        <v>589</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="1.143700787401575" bottom="1.143700787401575" header="0.75" footer="0.75"/>
-  <pageSetup paperSize="0" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated cci product files
</commit_message>
<xml_diff>
--- a/data/cci/cci-product.xlsx
+++ b/data/cci/cci-product.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stfc365-my.sharepoint.com/personal/alison_waterfall_stfc_ac_uk/Documents/Documents/GitHub/cci-vocabularies/data/cci/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="142" documentId="13_ncr:1_{8698D110-CEA0-44F5-A4A0-4B424D64BB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8AE1811C-B940-4021-823D-619C586D6182}"/>
+  <xr:revisionPtr revIDLastSave="147" documentId="13_ncr:1_{8698D110-CEA0-44F5-A4A0-4B424D64BB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA4398A5-DA59-4E3D-A681-45DF4C1F3D36}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-60" windowWidth="38640" windowHeight="21120" xr2:uid="{04DF87AA-227F-E848-BF0E-6E7C9BB1D368}"/>
+    <workbookView xWindow="38400" yWindow="2115" windowWidth="28800" windowHeight="15285" xr2:uid="{04DF87AA-227F-E848-BF0E-6E7C9BB1D368}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="591">
   <si>
     <t>URI</t>
   </si>
@@ -1787,6 +1787,9 @@
   </si>
   <si>
     <t>HMWR9-0.05deg_1MONTHLY</t>
+  </si>
+  <si>
+    <t>prod_hmwr9</t>
   </si>
   <si>
     <t>HMWR9-0.05deg</t>
@@ -8990,10 +8993,10 @@
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A252" s="2" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
   </sheetData>

</xml_diff>